<commit_message>
add: Cambio en los secuencias de docuemtos, se generarn automaticamente.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/Terceros Original.xlsx
+++ b/api/src/main/resources/importaciones/Terceros Original.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D46F94-76DC-4C28-92BE-684ECA8A72CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A2D87D-13D9-46EC-87E6-1C85F18F8363}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="120" windowWidth="18915" windowHeight="8475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="193">
   <si>
     <t>tipoIdentificacion</t>
   </si>
@@ -479,13 +479,133 @@
   </si>
   <si>
     <t>M</t>
+  </si>
+  <si>
+    <t>Codigo Salario</t>
+  </si>
+  <si>
+    <t>Codigo Establecimiento</t>
+  </si>
+  <si>
+    <t>Aplica Convenio</t>
+  </si>
+  <si>
+    <t>Tipo Discapacidad</t>
+  </si>
+  <si>
+    <t>Porcentaje Discapacidad</t>
+  </si>
+  <si>
+    <t>Tipo Identificacion Discapacidad</t>
+  </si>
+  <si>
+    <t>Identificacion Discapacidad</t>
+  </si>
+  <si>
+    <t>Beneficio Provincia Galapagos</t>
+  </si>
+  <si>
+    <t>Enfermedad Catastrófica</t>
+  </si>
+  <si>
+    <t>Codigo Residencia</t>
+  </si>
+  <si>
+    <t>Jaime Ismael</t>
+  </si>
+  <si>
+    <t>Juan Esteban</t>
+  </si>
+  <si>
+    <t>Ximena Alexandra</t>
+  </si>
+  <si>
+    <t>Kelly Daniela</t>
+  </si>
+  <si>
+    <t>Apellidos</t>
+  </si>
+  <si>
+    <t>Nombres</t>
+  </si>
+  <si>
+    <t>Boada Boada</t>
+  </si>
+  <si>
+    <t>Perez Perez</t>
+  </si>
+  <si>
+    <t>Paez Figueroa</t>
+  </si>
+  <si>
+    <t>Pazmiño Salas</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>Es Trabajador</t>
+  </si>
+  <si>
+    <t>24 de julio y 17 de septiembre</t>
+  </si>
+  <si>
+    <t>por ahi</t>
+  </si>
+  <si>
+    <t>av el inca y versalles</t>
+  </si>
+  <si>
+    <t>av del maestro y 6 de mrazo</t>
+  </si>
+  <si>
+    <t>0999999999</t>
+  </si>
+  <si>
+    <t>nnnn@hotmail.com</t>
+  </si>
+  <si>
+    <t>juanperez@hotmail.com</t>
+  </si>
+  <si>
+    <t>ximenapaez@hotmail.com</t>
+  </si>
+  <si>
+    <t>kellypazmino@hotmail.com</t>
+  </si>
+  <si>
+    <t>1751136138001</t>
+  </si>
+  <si>
+    <t>1751126138001</t>
+  </si>
+  <si>
+    <t>1751134138001</t>
+  </si>
+  <si>
+    <t>1751136108001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -520,8 +640,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -531,6 +659,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -566,7 +706,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -580,6 +720,12 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -987,56 +1133,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:AH28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.7109375" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="33.7109375" customWidth="1"/>
-    <col min="6" max="6" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.85546875" customWidth="1"/>
+    <col min="5" max="5" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" customWidth="1"/>
+    <col min="10" max="10" width="33.7109375" customWidth="1"/>
     <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.42578125" customWidth="1"/>
     <col min="13" max="13" width="17.42578125" customWidth="1"/>
     <col min="14" max="14" width="21.85546875" customWidth="1"/>
     <col min="15" max="16" width="21.85546875" style="1" customWidth="1"/>
-    <col min="17" max="19" width="21.85546875" customWidth="1"/>
-    <col min="20" max="21" width="17.7109375" customWidth="1"/>
+    <col min="17" max="31" width="21.85546875" customWidth="1"/>
+    <col min="32" max="33" width="17.7109375" customWidth="1"/>
+    <col min="34" max="34" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>128</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>127</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="15" t="s">
         <v>2</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>8</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>3</v>
@@ -1065,14 +1212,53 @@
       <c r="S1" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="U1" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="V1" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="W1" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="X1" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y1" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="Z1" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="AA1" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="AB1" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="AC1" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="AD1" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="AF1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>118</v>
       </c>
+      <c r="AH1" s="14" t="s">
+        <v>179</v>
+      </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1085,23 +1271,23 @@
       <c r="D2" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="K2" t="s">
         <v>11</v>
@@ -1130,36 +1316,51 @@
       <c r="S2" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="T2" t="s">
-        <v>115</v>
-      </c>
-      <c r="U2" t="s">
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>130</v>
       </c>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I3" t="s">
         <v>100</v>
       </c>
       <c r="L3" t="s">
@@ -1177,36 +1378,39 @@
       <c r="P3" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="T3" t="s">
-        <v>115</v>
-      </c>
-      <c r="U3" t="s">
-        <v>115</v>
+      <c r="AF3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>131</v>
       </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
       <c r="F4" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="H4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" t="s">
         <v>99</v>
       </c>
       <c r="L4" t="s">
@@ -1224,36 +1428,39 @@
       <c r="P4" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T4" t="s">
-        <v>116</v>
-      </c>
-      <c r="U4" t="s">
-        <v>115</v>
+      <c r="AF4" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>132</v>
       </c>
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="H5" t="s">
-        <v>84</v>
-      </c>
-      <c r="I5" t="s">
         <v>101</v>
       </c>
       <c r="L5" t="s">
@@ -1271,36 +1478,39 @@
       <c r="P5" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T5" t="s">
-        <v>115</v>
-      </c>
-      <c r="U5" t="s">
+      <c r="AF5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>133</v>
       </c>
+      <c r="E6" t="s">
+        <v>113</v>
+      </c>
       <c r="F6" t="s">
-        <v>113</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="H6" t="s">
-        <v>85</v>
-      </c>
-      <c r="I6" t="s">
         <v>102</v>
       </c>
       <c r="L6" t="s">
@@ -1327,36 +1537,51 @@
       <c r="S6" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="T6" t="s">
-        <v>115</v>
-      </c>
-      <c r="U6" t="s">
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="10"/>
+      <c r="Z6" s="10"/>
+      <c r="AA6" s="10"/>
+      <c r="AB6" s="10"/>
+      <c r="AC6" s="10"/>
+      <c r="AD6" s="10"/>
+      <c r="AE6" s="10"/>
+      <c r="AF6" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH6" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>134</v>
       </c>
+      <c r="E7" t="s">
+        <v>61</v>
+      </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="G7" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" t="s">
         <v>103</v>
       </c>
       <c r="L7" t="s">
@@ -1374,36 +1599,39 @@
       <c r="P7" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T7" t="s">
-        <v>116</v>
-      </c>
-      <c r="U7" t="s">
-        <v>115</v>
+      <c r="AF7" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>135</v>
       </c>
+      <c r="E8" t="s">
+        <v>62</v>
+      </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H8" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" t="s">
         <v>104</v>
       </c>
       <c r="L8" t="s">
@@ -1421,36 +1649,39 @@
       <c r="P8" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T8" t="s">
-        <v>115</v>
-      </c>
-      <c r="U8" t="s">
+      <c r="AF8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH8" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>136</v>
       </c>
+      <c r="E9" t="s">
+        <v>63</v>
+      </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="G9" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H9" t="s">
-        <v>88</v>
-      </c>
-      <c r="I9" t="s">
         <v>105</v>
       </c>
       <c r="L9" t="s">
@@ -1468,36 +1699,39 @@
       <c r="P9" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T9" t="s">
-        <v>116</v>
-      </c>
-      <c r="U9" t="s">
-        <v>115</v>
+      <c r="AF9" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>137</v>
       </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H10" t="s">
-        <v>89</v>
-      </c>
-      <c r="I10" t="s">
         <v>106</v>
       </c>
       <c r="L10" t="s">
@@ -1524,36 +1758,51 @@
       <c r="S10" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="T10" t="s">
-        <v>115</v>
-      </c>
-      <c r="U10" t="s">
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="10"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH10" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>47</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F11" t="s">
+      <c r="E11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>19</v>
       </c>
+      <c r="G11" t="s">
+        <v>90</v>
+      </c>
       <c r="H11" t="s">
-        <v>90</v>
-      </c>
-      <c r="I11" t="s">
         <v>107</v>
       </c>
       <c r="L11" t="s">
@@ -1571,36 +1820,39 @@
       <c r="P11" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T11" t="s">
-        <v>116</v>
-      </c>
-      <c r="U11" t="s">
-        <v>115</v>
+      <c r="AF11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="16" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="E12" t="s">
+        <v>66</v>
+      </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>91</v>
       </c>
       <c r="H12" t="s">
-        <v>91</v>
-      </c>
-      <c r="I12" t="s">
         <v>75</v>
       </c>
       <c r="L12" t="s">
@@ -1618,36 +1870,39 @@
       <c r="P12" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T12" t="s">
-        <v>115</v>
-      </c>
-      <c r="U12" t="s">
+      <c r="AF12" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH12" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="E13" t="s">
+        <v>67</v>
+      </c>
       <c r="F13" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="H13" t="s">
-        <v>92</v>
-      </c>
-      <c r="I13" t="s">
         <v>75</v>
       </c>
       <c r="L13" t="s">
@@ -1665,36 +1920,39 @@
       <c r="P13" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T13" t="s">
-        <v>115</v>
-      </c>
-      <c r="U13" t="s">
+      <c r="AF13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH13" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>141</v>
       </c>
+      <c r="E14" t="s">
+        <v>68</v>
+      </c>
       <c r="F14" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="H14" t="s">
-        <v>93</v>
-      </c>
-      <c r="I14" t="s">
         <v>108</v>
       </c>
       <c r="L14" t="s">
@@ -1721,36 +1979,51 @@
       <c r="S14" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="T14" t="s">
-        <v>115</v>
-      </c>
-      <c r="U14" t="s">
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="10"/>
+      <c r="Y14" s="10"/>
+      <c r="Z14" s="10"/>
+      <c r="AA14" s="10"/>
+      <c r="AB14" s="10"/>
+      <c r="AC14" s="10"/>
+      <c r="AD14" s="10"/>
+      <c r="AE14" s="10"/>
+      <c r="AF14" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH14" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>142</v>
       </c>
+      <c r="E15" t="s">
+        <v>69</v>
+      </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="H15" t="s">
-        <v>75</v>
-      </c>
-      <c r="I15" t="s">
         <v>109</v>
       </c>
       <c r="L15" t="s">
@@ -1768,38 +2041,41 @@
       <c r="P15" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T15" t="s">
-        <v>116</v>
-      </c>
-      <c r="U15" t="s">
-        <v>115</v>
+      <c r="AF15" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>52</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>143</v>
       </c>
+      <c r="E16" t="s">
+        <v>113</v>
+      </c>
       <c r="F16" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H16" t="s">
         <v>75</v>
       </c>
-      <c r="I16" t="s">
-        <v>75</v>
-      </c>
       <c r="L16" t="s">
         <v>119</v>
       </c>
@@ -1815,36 +2091,39 @@
       <c r="P16" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T16" t="s">
-        <v>115</v>
-      </c>
-      <c r="U16" t="s">
+      <c r="AF16" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH16" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
         <v>53</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>144</v>
       </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>19</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
-      </c>
-      <c r="I17" t="s">
         <v>75</v>
       </c>
       <c r="L17" t="s">
@@ -1862,36 +2141,39 @@
       <c r="P17" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T17" t="s">
-        <v>115</v>
-      </c>
-      <c r="U17" t="s">
+      <c r="AF17" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH17" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>145</v>
       </c>
+      <c r="E18" t="s">
+        <v>71</v>
+      </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="G18" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="H18" t="s">
-        <v>95</v>
-      </c>
-      <c r="I18" t="s">
         <v>75</v>
       </c>
       <c r="L18" t="s">
@@ -1909,36 +2191,39 @@
       <c r="P18" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T18" t="s">
-        <v>115</v>
-      </c>
-      <c r="U18" t="s">
-        <v>115</v>
+      <c r="AF18" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>55</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>146</v>
       </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="G19" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="H19" t="s">
-        <v>96</v>
-      </c>
-      <c r="I19" t="s">
         <v>110</v>
       </c>
       <c r="L19" t="s">
@@ -1956,36 +2241,39 @@
       <c r="P19" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T19" t="s">
-        <v>115</v>
-      </c>
-      <c r="U19" t="s">
+      <c r="AF19" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH19" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>147</v>
       </c>
+      <c r="E20" t="s">
+        <v>73</v>
+      </c>
       <c r="F20" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>19</v>
+        <v>97</v>
       </c>
       <c r="H20" t="s">
-        <v>97</v>
-      </c>
-      <c r="I20" t="s">
         <v>111</v>
       </c>
       <c r="L20" t="s">
@@ -2003,36 +2291,39 @@
       <c r="P20" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T20" t="s">
-        <v>115</v>
-      </c>
-      <c r="U20" t="s">
-        <v>115</v>
+      <c r="AF20" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>38</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>57</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>148</v>
       </c>
+      <c r="E21" t="s">
+        <v>74</v>
+      </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="G21" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="H21" t="s">
-        <v>98</v>
-      </c>
-      <c r="I21" t="s">
         <v>112</v>
       </c>
       <c r="L21" t="s">
@@ -2050,18 +2341,336 @@
       <c r="P21" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="T21" t="s">
-        <v>115</v>
-      </c>
-      <c r="U21" t="s">
-        <v>116</v>
-      </c>
+      <c r="AF21" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E22" t="s">
+        <v>180</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="L22" t="s">
+        <v>116</v>
+      </c>
+      <c r="M22">
+        <v>593</v>
+      </c>
+      <c r="N22" s="7">
+        <v>17</v>
+      </c>
+      <c r="O22" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P22" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="T22" t="s">
+        <v>169</v>
+      </c>
+      <c r="U22" t="s">
+        <v>163</v>
+      </c>
+      <c r="V22">
+        <v>4</v>
+      </c>
+      <c r="W22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="X22" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y22" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>116</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E23" t="s">
+        <v>181</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L23" t="s">
+        <v>116</v>
+      </c>
+      <c r="M23">
+        <v>593</v>
+      </c>
+      <c r="N23" s="7">
+        <v>17</v>
+      </c>
+      <c r="O23" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P23" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="T23" t="s">
+        <v>170</v>
+      </c>
+      <c r="U23" t="s">
+        <v>164</v>
+      </c>
+      <c r="V23">
+        <v>7</v>
+      </c>
+      <c r="W23" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="X23" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y23" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z23">
+        <v>10</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB23">
+        <v>1234567890</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>116</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE23" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>171</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E24" t="s">
+        <v>182</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="L24" t="s">
+        <v>116</v>
+      </c>
+      <c r="M24">
+        <v>593</v>
+      </c>
+      <c r="N24" s="7">
+        <v>17</v>
+      </c>
+      <c r="O24" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P24" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="T24" t="s">
+        <v>171</v>
+      </c>
+      <c r="U24" t="s">
+        <v>165</v>
+      </c>
+      <c r="V24">
+        <v>5</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="X24" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y24" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>116</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE24" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E25" t="s">
+        <v>183</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="L25" t="s">
+        <v>116</v>
+      </c>
+      <c r="M25">
+        <v>593</v>
+      </c>
+      <c r="N25" s="7">
+        <v>17</v>
+      </c>
+      <c r="O25" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P25" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="T25" t="s">
+        <v>172</v>
+      </c>
+      <c r="U25" t="s">
+        <v>166</v>
+      </c>
+      <c r="V25">
+        <v>8</v>
+      </c>
+      <c r="W25" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="X25" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y25" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z25">
+        <v>75</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB25">
+        <v>987654321</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>116</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE25" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="L26" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="O28"/>
+      <c r="P28"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{78F473DD-69A3-426A-B9CD-5774C24736D8}"/>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{78F473DD-69A3-426A-B9CD-5774C24736D8}"/>
+    <hyperlink ref="I22" r:id="rId2" xr:uid="{F6598700-3944-46FB-9422-D9A763A2C35C}"/>
+    <hyperlink ref="I23" r:id="rId3" xr:uid="{FC2BD439-7F5F-4490-B853-9AD50D71DEF3}"/>
+    <hyperlink ref="I24" r:id="rId4" xr:uid="{59004BDF-3D99-4D14-A8B2-5F405956BC79}"/>
+    <hyperlink ref="I25" r:id="rId5" xr:uid="{486C6CE2-ADA6-4141-A430-643C72E4D8AF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add: Retencion en Talon Resumen, y Correcion del Logo del pdf en los documentos.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/Terceros Original.xlsx
+++ b/api/src/main/resources/importaciones/Terceros Original.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A2D87D-13D9-46EC-87E6-1C85F18F8363}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB90481B-6C10-44F5-A85A-A132D637A340}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="120" windowWidth="18915" windowHeight="8475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="193">
   <si>
     <t>tipoIdentificacion</t>
   </si>
@@ -2361,6 +2361,9 @@
       <c r="C22" s="1" t="s">
         <v>189</v>
       </c>
+      <c r="D22" s="1" t="s">
+        <v>148</v>
+      </c>
       <c r="E22" t="s">
         <v>180</v>
       </c>
@@ -2432,6 +2435,9 @@
       <c r="C23" s="1" t="s">
         <v>190</v>
       </c>
+      <c r="D23" s="1" t="s">
+        <v>148</v>
+      </c>
       <c r="E23" t="s">
         <v>181</v>
       </c>
@@ -2512,6 +2518,9 @@
       <c r="C24" s="1" t="s">
         <v>191</v>
       </c>
+      <c r="D24" s="1" t="s">
+        <v>148</v>
+      </c>
       <c r="E24" t="s">
         <v>182</v>
       </c>
@@ -2582,6 +2591,9 @@
       </c>
       <c r="C25" s="1" t="s">
         <v>192</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="E25" t="s">
         <v>183</v>

</xml_diff>